<commit_message>
Configure Render Earth Engine deployment
</commit_message>
<xml_diff>
--- a/timeseries_data.xlsx
+++ b/timeseries_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,63 +430,63 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>35.92</v>
+        <v>35.52</v>
       </c>
       <c r="B2" t="n">
-        <v>0.143</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>41.91</v>
+        <v>37.24</v>
       </c>
       <c r="B3" t="n">
-        <v>0.145</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>31.04</v>
+        <v>37.95</v>
       </c>
       <c r="B4" t="n">
-        <v>0.201</v>
+        <v>0.203</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>45.91</v>
+        <v>37.56</v>
       </c>
       <c r="B5" t="n">
-        <v>0.224</v>
+        <v>0.158</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>38.7</v>
+        <v>36.55</v>
       </c>
       <c r="B6" t="n">
-        <v>0.178</v>
+        <v>0.188</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>38.7</v>
+        <v>42.67</v>
       </c>
       <c r="B7" t="n">
-        <v>0.178</v>
+        <v>0.152</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>38.7</v>
+        <v>37.33</v>
       </c>
       <c r="B8" t="n">
-        <v>0.178</v>
+        <v>0.168</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>38.7</v>
+        <v>37.23</v>
       </c>
       <c r="B9" t="n">
         <v>0.178</v>
@@ -494,178 +494,26 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>38.7</v>
+        <v>36.71</v>
       </c>
       <c r="B10" t="n">
-        <v>0.178</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>38.7</v>
+        <v>38.22</v>
       </c>
       <c r="B11" t="n">
-        <v>0.178</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>33.84</v>
+        <v>38.55</v>
       </c>
       <c r="B12" t="n">
-        <v>0.26</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>34</v>
-      </c>
-      <c r="B13" t="n">
-        <v>0.192</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>37.82</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0.146</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>39.12</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.114</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>42.81</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0.172</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="B17" t="n">
-        <v>0.178</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="B18" t="n">
-        <v>0.178</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.178</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.178</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.178</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="B22" t="n">
-        <v>0.178</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>36.03</v>
-      </c>
-      <c r="B23" t="n">
-        <v>0.333</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>36.31</v>
-      </c>
-      <c r="B24" t="n">
-        <v>0.259</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>35.14</v>
-      </c>
-      <c r="B25" t="n">
-        <v>0.173</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>37.91</v>
-      </c>
-      <c r="B26" t="n">
-        <v>0.132</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>42.73</v>
-      </c>
-      <c r="B27" t="n">
-        <v>0.124</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="B28" t="n">
-        <v>0.143</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>42.06</v>
-      </c>
-      <c r="B29" t="n">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>37.23</v>
-      </c>
-      <c r="B30" t="n">
-        <v>0.254</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>38.51</v>
-      </c>
-      <c r="B31" t="n">
-        <v>0.183</v>
+        <v>0.156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>